<commit_message>
Restringe o escopo de mídia a listagem, sem produção
A skill lista os vídeos com página, rótulo, assunto e link, para que sejam
localizados depois. Não produz, não legenda, não dubla e não recomenda método de
produção — isso é decisão e execução da FEA.

Removida a coluna Método ES da planilha e a seção de recomendação de legenda,
dublagem ou regravação do anexo, substituída por nota de escopo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P3zqXZaMgjjVCZhfTEeo1A
</commit_message>
<xml_diff>
--- a/traducciones/relleno-ojeras/Inventario_Videos_QR_Olheiras.xlsx
+++ b/traducciones/relleno-ojeras/Inventario_Videos_QR_Olheiras.xlsx
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -659,7 +659,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -717,7 +716,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -784,7 +782,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -837,7 +834,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
@@ -852,9 +848,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
     <row r="26">
       <c r="A26" s="26" t="inlineStr">
         <is>
@@ -873,6 +866,20 @@
       <c r="A28" s="27" t="inlineStr">
         <is>
           <t>Coluna «Valor de referência»: foto do inventário conferido em 21/08/2026. Serve de conferência — se a fórmula divergir depois, é porque alguém editou as abas de dados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="26" t="inlineStr">
+        <is>
+          <t>Escopo desta planilha</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Listar e localizar os vídeos e seus links. A produção da versão em espanhol — legenda, dublagem ou regravação — é decisão e execução da FEA, fora do escopo deste inventário.</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2244,25 +2251,20 @@
       </c>
       <c r="J1" s="8" t="inlineStr">
         <is>
-          <t>Método ES</t>
+          <t>Link ES</t>
         </is>
       </c>
       <c r="K1" s="8" t="inlineStr">
         <is>
-          <t>Link ES</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="L1" s="8" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Responsável</t>
         </is>
       </c>
       <c r="M1" s="8" t="inlineStr">
-        <is>
-          <t>Responsável</t>
-        </is>
-      </c>
-      <c r="N1" s="8" t="inlineStr">
         <is>
           <t>Data prevista</t>
         </is>
@@ -2313,14 +2315,13 @@
         <v>1</v>
       </c>
       <c r="J2" s="10" t="n"/>
-      <c r="K2" s="10" t="n"/>
-      <c r="L2" s="10" t="inlineStr">
+      <c r="K2" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L2" s="10" t="n"/>
       <c r="M2" s="10" t="n"/>
-      <c r="N2" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
@@ -2367,14 +2368,13 @@
         <v>1</v>
       </c>
       <c r="J3" s="10" t="n"/>
-      <c r="K3" s="10" t="n"/>
-      <c r="L3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L3" s="10" t="n"/>
       <c r="M3" s="10" t="n"/>
-      <c r="N3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -2421,14 +2421,13 @@
         <v>1</v>
       </c>
       <c r="J4" s="10" t="n"/>
-      <c r="K4" s="10" t="n"/>
-      <c r="L4" s="10" t="inlineStr">
+      <c r="K4" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L4" s="10" t="n"/>
       <c r="M4" s="10" t="n"/>
-      <c r="N4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -2475,14 +2474,13 @@
         <v>1</v>
       </c>
       <c r="J5" s="10" t="n"/>
-      <c r="K5" s="10" t="n"/>
-      <c r="L5" s="10" t="inlineStr">
+      <c r="K5" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L5" s="10" t="n"/>
       <c r="M5" s="10" t="n"/>
-      <c r="N5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -2529,14 +2527,13 @@
         <v>1</v>
       </c>
       <c r="J6" s="10" t="n"/>
-      <c r="K6" s="10" t="n"/>
-      <c r="L6" s="10" t="inlineStr">
+      <c r="K6" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L6" s="10" t="n"/>
       <c r="M6" s="10" t="n"/>
-      <c r="N6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -2579,14 +2576,13 @@
         <v>1</v>
       </c>
       <c r="J7" s="10" t="n"/>
-      <c r="K7" s="10" t="n"/>
-      <c r="L7" s="10" t="inlineStr">
+      <c r="K7" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L7" s="10" t="n"/>
       <c r="M7" s="10" t="n"/>
-      <c r="N7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -2629,14 +2625,13 @@
         <v>1</v>
       </c>
       <c r="J8" s="10" t="n"/>
-      <c r="K8" s="10" t="n"/>
-      <c r="L8" s="10" t="inlineStr">
+      <c r="K8" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L8" s="10" t="n"/>
       <c r="M8" s="10" t="n"/>
-      <c r="N8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -2679,14 +2674,13 @@
         <v>1</v>
       </c>
       <c r="J9" s="10" t="n"/>
-      <c r="K9" s="10" t="n"/>
-      <c r="L9" s="10" t="inlineStr">
+      <c r="K9" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L9" s="10" t="n"/>
       <c r="M9" s="10" t="n"/>
-      <c r="N9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -2729,14 +2723,13 @@
         <v>2</v>
       </c>
       <c r="J10" s="10" t="n"/>
-      <c r="K10" s="10" t="n"/>
-      <c r="L10" s="10" t="inlineStr">
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L10" s="10" t="n"/>
       <c r="M10" s="10" t="n"/>
-      <c r="N10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -2779,14 +2772,13 @@
         <v>1</v>
       </c>
       <c r="J11" s="10" t="n"/>
-      <c r="K11" s="10" t="n"/>
-      <c r="L11" s="10" t="inlineStr">
+      <c r="K11" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L11" s="10" t="n"/>
       <c r="M11" s="10" t="n"/>
-      <c r="N11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -2829,14 +2821,13 @@
         <v>2</v>
       </c>
       <c r="J12" s="10" t="n"/>
-      <c r="K12" s="10" t="n"/>
-      <c r="L12" s="10" t="inlineStr">
+      <c r="K12" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L12" s="10" t="n"/>
       <c r="M12" s="10" t="n"/>
-      <c r="N12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -2879,14 +2870,13 @@
         <v>1</v>
       </c>
       <c r="J13" s="10" t="n"/>
-      <c r="K13" s="10" t="n"/>
-      <c r="L13" s="10" t="inlineStr">
+      <c r="K13" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L13" s="10" t="n"/>
       <c r="M13" s="10" t="n"/>
-      <c r="N13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -2929,14 +2919,13 @@
         <v>1</v>
       </c>
       <c r="J14" s="10" t="n"/>
-      <c r="K14" s="10" t="n"/>
-      <c r="L14" s="10" t="inlineStr">
+      <c r="K14" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L14" s="10" t="n"/>
       <c r="M14" s="10" t="n"/>
-      <c r="N14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -2979,14 +2968,13 @@
         <v>1</v>
       </c>
       <c r="J15" s="10" t="n"/>
-      <c r="K15" s="10" t="n"/>
-      <c r="L15" s="10" t="inlineStr">
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L15" s="10" t="n"/>
       <c r="M15" s="10" t="n"/>
-      <c r="N15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -3029,14 +3017,13 @@
         <v>1</v>
       </c>
       <c r="J16" s="10" t="n"/>
-      <c r="K16" s="10" t="n"/>
-      <c r="L16" s="10" t="inlineStr">
+      <c r="K16" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L16" s="10" t="n"/>
       <c r="M16" s="10" t="n"/>
-      <c r="N16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -3083,14 +3070,13 @@
         <v>1</v>
       </c>
       <c r="J17" s="10" t="n"/>
-      <c r="K17" s="10" t="n"/>
-      <c r="L17" s="10" t="inlineStr">
+      <c r="K17" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L17" s="10" t="n"/>
       <c r="M17" s="10" t="n"/>
-      <c r="N17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -3137,14 +3123,13 @@
         <v>1</v>
       </c>
       <c r="J18" s="10" t="n"/>
-      <c r="K18" s="10" t="n"/>
-      <c r="L18" s="10" t="inlineStr">
+      <c r="K18" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L18" s="10" t="n"/>
       <c r="M18" s="10" t="n"/>
-      <c r="N18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -3191,14 +3176,13 @@
         <v>1</v>
       </c>
       <c r="J19" s="10" t="n"/>
-      <c r="K19" s="10" t="n"/>
-      <c r="L19" s="10" t="inlineStr">
+      <c r="K19" s="10" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
+      <c r="L19" s="10" t="n"/>
       <c r="M19" s="10" t="n"/>
-      <c r="N19" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3669,6 +3653,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="18" t="inlineStr">
         <is>
@@ -3742,16 +3727,8 @@
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Método ES</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>legenda · dublagem · regravação</t>
-        </is>
-      </c>
+      <c r="A9" s="18" t="n"/>
+      <c r="B9" s="19" t="n"/>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
@@ -3777,6 +3754,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
         <is>
@@ -3833,16 +3811,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Método ES</t>
-        </is>
-      </c>
-      <c r="B18" s="21" t="inlineStr">
-        <is>
-          <t>legenda</t>
-        </is>
-      </c>
+      <c r="A18" s="3" t="n"/>
+      <c r="B18" s="21" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Adiciona aba com a lista completa dos 32 QR Codes
Aba «Todos os QR»: lista plana de todas as ocorrências, com página, tipo,
plataforma, rótulo, link completo, marcador de tempo, indicação de repetição e
coluna «Traduzir?» separando os 20 QR de vídeo dos 12 de artigo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P3zqXZaMgjjVCZhfTEeo1A
</commit_message>
<xml_diff>
--- a/traducciones/relleno-ojeras/Inventario_Videos_QR_Olheiras.xlsx
+++ b/traducciones/relleno-ojeras/Inventario_Videos_QR_Olheiras.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeos a traduzir" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ativos únicos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artigos (não traduzir)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Todos os QR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeos a traduzir" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ativos únicos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artigos (não traduzir)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -104,7 +105,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -129,6 +130,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="007F7F7F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -158,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -220,6 +231,30 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -894,6 +929,1355 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="72" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Pág.</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Rótulo / referência</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Link completo</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Marcador t= (s)</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>Repetido</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>Traduzir?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Artigo do próprio autor (JCEDR)</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1q9C5LiGEo1ytzX5z5Xybmb9gqkmzJEVp/view</t>
+        </is>
+      </c>
+      <c r="G2" s="28" t="n"/>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I2" s="30" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="31" t="n">
+        <v>12</v>
+      </c>
+      <c r="C3" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D3" s="31" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>E-book Allergan — Facial Aging Flipchart</t>
+        </is>
+      </c>
+      <c r="F3" s="31" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1fEV5ed5ht84TZMXfyFY0UQaepV1aVBxN/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="G3" s="31" t="n"/>
+      <c r="H3" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I3" s="32" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="28" t="n">
+        <v>13</v>
+      </c>
+      <c r="C4" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Krutmann 2017</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1gaeyIZq9FIraDHyogy4R3SPemwV6lZzu/view</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="n"/>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I4" s="30" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="31" t="n">
+        <v>13</v>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Freytag 2022 — biomecânica facial</t>
+        </is>
+      </c>
+      <c r="F5" s="31" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1nedzvMiWbnHCrsfiqUKZo3djmO5ryAMU/view</t>
+        </is>
+      </c>
+      <c r="G5" s="31" t="n"/>
+      <c r="H5" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I5" s="32" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="28" t="n">
+        <v>14</v>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Outros fatores que levam ao envelhecimento</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1HwoJC-1_lPVUSta0TDL_rTCL6s-zbfPP/view</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n"/>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I6" s="34" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="31" t="n">
+        <v>15</v>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D7" s="31" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Shaw 2011 — Aging of the Facial Skeleton</t>
+        </is>
+      </c>
+      <c r="F7" s="31" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1hHRSweDij0lvIhV6MnfH_Z4A5bzksbls/view</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="n"/>
+      <c r="H7" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I7" s="32" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="28" t="n">
+        <v>17</v>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Gierloff 2012 — Midfacial Fat Compartments</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1EZrxsmfLnASki1Xw-pj8mnOu2UE-2wED/view</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n"/>
+      <c r="H8" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I8" s="30" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="31" t="n">
+        <v>18</v>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D9" s="31" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Livro AFE (nome de arquivo ilegível)</t>
+        </is>
+      </c>
+      <c r="F9" s="31" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1KMqjjp5S5Vxe-x6dL3VFzyd3h2zL0TYa/view</t>
+        </is>
+      </c>
+      <c r="G9" s="31" t="n"/>
+      <c r="H9" s="31" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I9" s="32" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="28" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Anatomia no cadáver — revisão completa</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1zg1QC8ae2GOl4xOB5dWWArZBzKhfJHXk/view?t=30</t>
+        </is>
+      </c>
+      <c r="G10" s="34" t="n">
+        <v>30</v>
+      </c>
+      <c r="H10" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I10" s="34" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="31" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="31" t="n">
+        <v>22</v>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D11" s="31" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>O que é SOOF?</t>
+        </is>
+      </c>
+      <c r="F11" s="31" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1OmShQSqAWbdBPSBzhcjjnEGw0bh_XUbT/view</t>
+        </is>
+      </c>
+      <c r="G11" s="31" t="n"/>
+      <c r="H11" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I11" s="35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="28" t="n">
+        <v>25</v>
+      </c>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D12" s="28" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Livro AFE (repete pág. 18)</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1KMqjjp5S5Vxe-x6dL3VFzyd3h2zL0TYa/view</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n"/>
+      <c r="H12" s="28" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I12" s="30" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="31" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="31" t="n">
+        <v>28</v>
+      </c>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D13" s="31" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>PT 2. Anatomia dos ligamentos verdadeiros e falsos</t>
+        </is>
+      </c>
+      <c r="F13" s="31" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1is3EUbeHVE3KDhhZsX_LG6koR6uGZY31/view</t>
+        </is>
+      </c>
+      <c r="G13" s="31" t="n"/>
+      <c r="H13" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I13" s="35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="28" t="n">
+        <v>30</v>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Livro AFE (repete pág. 18)</t>
+        </is>
+      </c>
+      <c r="F14" s="28" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1KMqjjp5S5Vxe-x6dL3VFzyd3h2zL0TYa/view</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n"/>
+      <c r="H14" s="28" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I14" s="30" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="31" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="31" t="n">
+        <v>34</v>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>PT 1. Anatomia dos ligamentos verdadeiros e falsos</t>
+        </is>
+      </c>
+      <c r="F15" s="31" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1PwikjaqDastNx9AR9pqqH-OHxGqWHM7g/view</t>
+        </is>
+      </c>
+      <c r="G15" s="31" t="n"/>
+      <c r="H15" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I15" s="35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="28" t="n">
+        <v>42</v>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D16" s="28" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>de la Guardia — reologia do AH</t>
+        </is>
+      </c>
+      <c r="F16" s="28" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1AzTX83z4wetiAroor7GvT4i8jWsE1LB3/view</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n"/>
+      <c r="H16" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I16" s="30" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="31" t="n">
+        <v>42</v>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D17" s="31" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Swelling factor</t>
+        </is>
+      </c>
+      <c r="F17" s="31" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1Bx2WTa_isjzuzG7kFRbJatKmiWwDQU5B/view</t>
+        </is>
+      </c>
+      <c r="G17" s="31" t="n"/>
+      <c r="H17" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I17" s="32" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="28" t="n">
+        <v>46</v>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D18" s="28" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Reologia</t>
+        </is>
+      </c>
+      <c r="F18" s="28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=E6Jr5bm__Ys</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n"/>
+      <c r="H18" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I18" s="34" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="31" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="31" t="n">
+        <v>49</v>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Planejamento de preenchimento</t>
+        </is>
+      </c>
+      <c r="F19" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/shorts/PkKmtkkbV14</t>
+        </is>
+      </c>
+      <c r="G19" s="31" t="n"/>
+      <c r="H19" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I19" s="35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="28" t="n">
+        <v>49</v>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D20" s="28" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Pertuitos e raciocínio clínico</t>
+        </is>
+      </c>
+      <c r="F20" s="28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/shorts/kbocfP1toT4</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n"/>
+      <c r="H20" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I20" s="34" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="31" t="n">
+        <v>49</v>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D21" s="31" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Marcação dos ligamentos</t>
+        </is>
+      </c>
+      <c r="F21" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/shorts/l05fBSo_5ws</t>
+        </is>
+      </c>
+      <c r="G21" s="31" t="n"/>
+      <c r="H21" s="31" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I21" s="35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="C22" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D22" s="28" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Explicação do planejamento dos pertuitos</t>
+        </is>
+      </c>
+      <c r="F22" s="28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/shorts/awa6wCo_Zl8</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n"/>
+      <c r="H22" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I22" s="34" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="31" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="31" t="n">
+        <v>51</v>
+      </c>
+      <c r="C23" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D23" s="31" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Primeiro pertuito</t>
+        </is>
+      </c>
+      <c r="F23" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=63nh2AQiAtA</t>
+        </is>
+      </c>
+      <c r="G23" s="31" t="n"/>
+      <c r="H23" s="31" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I23" s="35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="28" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="28" t="n">
+        <v>51</v>
+      </c>
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D24" s="28" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Segundo pertuito</t>
+        </is>
+      </c>
+      <c r="F24" s="28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GX9u2yyem7E</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n"/>
+      <c r="H24" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I24" s="34" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="31" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="31" t="n">
+        <v>52</v>
+      </c>
+      <c r="C25" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Terceiro e quarto pertuito</t>
+        </is>
+      </c>
+      <c r="F25" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=FHyZ4Ee_q1E</t>
+        </is>
+      </c>
+      <c r="G25" s="31" t="n"/>
+      <c r="H25" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I25" s="35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="28" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="28" t="n">
+        <v>54</v>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D26" s="28" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Demonstração do botão anestésico</t>
+        </is>
+      </c>
+      <c r="F26" s="28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/shorts/CrQ3cQIpKpc</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n"/>
+      <c r="H26" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I26" s="34" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="31" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="31" t="n">
+        <v>57</v>
+      </c>
+      <c r="C27" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>Técnica completa / raciocínio clínico</t>
+        </is>
+      </c>
+      <c r="F27" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/shorts/_UvdKBkx3dU</t>
+        </is>
+      </c>
+      <c r="G27" s="31" t="n"/>
+      <c r="H27" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I27" s="35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="28" t="n">
+        <v>57</v>
+      </c>
+      <c r="C28" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D28" s="28" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Marcação dos ligamentos (repete pág. 49)</t>
+        </is>
+      </c>
+      <c r="F28" s="28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/shorts/l05fBSo_5ws</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n"/>
+      <c r="H28" s="28" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I28" s="34" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="31" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="31" t="n">
+        <v>57</v>
+      </c>
+      <c r="C29" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D29" s="31" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>Primeiro pertuito (repete pág. 51)</t>
+        </is>
+      </c>
+      <c r="F29" s="31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=63nh2AQiAtA</t>
+        </is>
+      </c>
+      <c r="G29" s="31" t="n"/>
+      <c r="H29" s="31" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I29" s="35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="28" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="28" t="n">
+        <v>58</v>
+      </c>
+      <c r="C30" s="29" t="inlineStr">
+        <is>
+          <t>Artigo/PDF</t>
+        </is>
+      </c>
+      <c r="D30" s="28" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Kato 2022 (JOCD) — tear trough</t>
+        </is>
+      </c>
+      <c r="F30" s="28" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1_hzAqkbwOV5hdJL__os_-2jS16KYEWh1/view</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n"/>
+      <c r="H30" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I30" s="30" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="31" t="n">
+        <v>61</v>
+      </c>
+      <c r="C31" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D31" s="31" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Hialuronidase na região orbital — caso clínico 2</t>
+        </is>
+      </c>
+      <c r="F31" s="31" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/18J0kJ0kq_OiVoL7ExuHxsQJZG_DzysLS/view?t=1100</t>
+        </is>
+      </c>
+      <c r="G31" s="35" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H31" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I31" s="35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="28" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="28" t="n">
+        <v>61</v>
+      </c>
+      <c r="C32" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D32" s="28" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>Hialuronidase na região orbital — aula 8</t>
+        </is>
+      </c>
+      <c r="F32" s="28" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1o8GJ5chWVE3bAnvLYUbzfBo5Lqw7v95Z/view?t=94</t>
+        </is>
+      </c>
+      <c r="G32" s="34" t="n">
+        <v>94</v>
+      </c>
+      <c r="H32" s="28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I32" s="34" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="31" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="31" t="n">
+        <v>64</v>
+      </c>
+      <c r="C33" s="33" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="D33" s="31" t="inlineStr">
+        <is>
+          <t>Google Drive</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>Raciocínio clínico para evitar irregularidades e relevo</t>
+        </is>
+      </c>
+      <c r="F33" s="31" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1cKZXapLdvwJ-YPATGMQPOBvqyX9mrn2L/view?t=164</t>
+        </is>
+      </c>
+      <c r="G33" s="35" t="n">
+        <v>164</v>
+      </c>
+      <c r="H33" s="31" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I33" s="35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>32 QR Codes decodificados do PDF (OpenCV 300/450 dpi). 20 apontam para vídeo, 12 para artigo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Coluna «Traduzir?»: SIM = precisa de versão ES e o QR terá de ser regerado. NÃO = artigo científico, permanece em inglês e o QR não muda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Coluna «Marcador t=»: em vermelho, o link abre o vídeo num ponto específico — recalcular se a versão ES tiver corte diferente.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2178,7 +3562,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3189,7 +4573,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3633,7 +5017,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3653,7 +5037,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="18" t="inlineStr">
         <is>
@@ -3754,7 +5137,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
         <is>

</xml_diff>